<commit_message>
Final update for deployment
</commit_message>
<xml_diff>
--- a/reports/GST_Reconciliation_Report.xlsx
+++ b/reports/GST_Reconciliation_Report.xlsx
@@ -1,13 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice Register" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation Report" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,7 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="₹#,##0.00"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -27,17 +31,42 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +74,20 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,455 +453,587 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Invoice Number</t>
+          <t>invoice_number</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>GSTIN</t>
+          <t>supplier_gstin</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>buyer_gstin</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Invoice Type</t>
+          <t>vendor_name</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Taxable Value (₹)</t>
+          <t>date</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Tax Amount (₹)</t>
+          <t>taxable_value</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Total Amount (₹)</t>
+          <t>tax_amount</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>total_amount</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Confidence Score</t>
+          <t>filing_period</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Uploaded At</t>
+          <t>status</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>INV/2024/001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>NOT_FOUND</t>
+          <t>27AAACD1234A1Z5</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>27BBBCD5678B1Z2</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>purchase</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Missing in Portal</t>
-        </is>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>2026-04-17 10:21:43</t>
+          <t>TATA MOTORS LTD</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>15-04-2024</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>100000</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>18000</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>118000</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>April 2024</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Matched</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>AMZ-9901</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NOT_FOUND</t>
+          <t>29AAACA1234A1Z5</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>27AAACD1234A1Z5</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>purchase</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Missing in Portal</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>2026-04-17 10:33:22</t>
+          <t>AMAZON SELLER SERVICES</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>10-05-2024</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>3600</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>23600</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>May 2024</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>LOCAL-STORE-01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NOT_FOUND</t>
+          <t>27MMMAD1234A1Z5</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>10.32.0000</t>
+          <t>27AAACD1234A1Z5</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>purchase</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="inlineStr">
+          <t>MODERN STATIONERY</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>12-05-2024</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>5250</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>May 2024</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>Missing in Portal</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>2026-04-23 03:42:06</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>REL/MAY/992</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NOT_FOUND</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>10.32.0000</t>
+          <t>07AAACR1234R1Z1</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>purchase</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
+          <t>RETAIL</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>05/05/2024</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>6000</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>May 2024 → Q1 FY2024-25</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Missing in Portal</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="86" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>invoice_number</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>gstin</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>taxable_value</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>external_taxable</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tax_amount</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>external_tax</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>tax_difference</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>INV/2024/001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>27AAACD1234A1Z5</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>18000</v>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Invoice matches GST portal records perfectly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AMZ-9901</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>29AAACA1234A1Z5</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>3600</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>3100</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Tax amount differs by ₹500.00. Verify with your CA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>LOCAL-STORE-01</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>27MMMAD1234A1Z5</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v/>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Missing in Portal</t>
         </is>
       </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>2026-04-23 16:16:44</t>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Invoice found in your books but absent from GST portal. May indicate delayed filing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>REL/MAY/992</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>07AAACR1234R1Z1</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v/>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Missing in Portal</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Invoice found in your books but absent from GST portal. May indicate delayed filing.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>MISC/882</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NOT_FOUND</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>purchase</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
+          <t>07AAACR1234R1Z1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Missing in Portal</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>2026-04-24 03:36:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>NOT_FOUND</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>purchase</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Missing in Portal</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>2026-04-24 03:42:57</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>INV-101</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>27ABCDE1234F1Z5</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>purchase</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1800</v>
-      </c>
-      <c r="G8" t="n">
-        <v>11800</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Matched</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>2026-04-24 03:44:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>INV-102</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>09PQRST5678G2Z1</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>purchase</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>4661.02</v>
-      </c>
-      <c r="F9" t="n">
-        <v>838.98</v>
-      </c>
-      <c r="G9" t="n">
-        <v>5500</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Mismatch</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>2026-04-24 03:45:39</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>INV-101</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>27ABCDE1234F1Z5</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>purchase</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F10" t="n">
-        <v>1800</v>
-      </c>
-      <c r="G10" t="n">
-        <v>11800</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Matched</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>2026-04-24 03:47:32</t>
-        </is>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Missing in Books</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>GST portal has this invoice but it has not been uploaded to the system.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Total Invoices</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Total Tax</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>21862</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Status: Matched</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Status: Mismatch</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Status: Missing in Portal</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: initial production-ready GST Helper.AI with Tally integration
</commit_message>
<xml_diff>
--- a/reports/GST_Reconciliation_Report.xlsx
+++ b/reports/GST_Reconciliation_Report.xlsx
@@ -49,12 +49,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
         <bgColor rgb="00FFC7CE"/>
       </patternFill>
@@ -63,6 +57,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
         <bgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -464,7 +464,7 @@
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -562,7 +562,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Matched</t>
+          <t>Mismatch</t>
         </is>
       </c>
     </row>
@@ -606,7 +606,7 @@
           <t>May 2024</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Mismatch</t>
         </is>
@@ -652,7 +652,7 @@
           <t>May 2024</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Missing in Portal</t>
         </is>
@@ -693,7 +693,171 @@
           <t>May 2024 → Q1 FY2024-25</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Missing in Portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>INV/2024/001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>27AAACD1234A1Z5</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>TATA MOTORS LTD</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>15-04-2024</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>9000</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>April 2024 → Q1 FY2024-25</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>INV/2024/001</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>27AAACD1234A1Z5</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>TATA MOTORS LTD</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>15-04-2024</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>9000</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>April 2024 → Q1 FY2024-25</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>REL/MAY/992</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07AAACR1234R1Z1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>RETAIL</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>05/05/2024</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>6000</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>May 2024 → Q1 FY2024-25</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Missing in Portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>REL/MAY/992</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>07AAACR1234R1Z1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>RETAIL</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>05/05/2024</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>6000</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>May 2024 → Q1 FY2024-25</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
         <is>
           <t>Missing in Portal</t>
         </is>
@@ -710,7 +874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -721,7 +885,7 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="86" customWidth="1" min="9" max="9"/>
+    <col width="92" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -797,7 +961,7 @@
       <c r="G2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>Matched</t>
         </is>
@@ -834,7 +998,7 @@
       <c r="G3" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Mismatch</t>
         </is>
@@ -871,7 +1035,7 @@
       <c r="G4" s="2" t="n">
         <v>250</v>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Missing in Portal</t>
         </is>
@@ -908,7 +1072,7 @@
       <c r="G5" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Missing in Portal</t>
         </is>
@@ -922,35 +1086,183 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>INV/2024/001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>27AAACD1234A1Z5</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>18000</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>-18000</v>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Taxable value differs by ₹100000.00; Tax amount differs by ₹18000.00. Verify with your CA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>INV/2024/001</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>27AAACD1234A1Z5</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>18000</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>-18000</v>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Taxable value differs by ₹100000.00; Tax amount differs by ₹18000.00. Verify with your CA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>REL/MAY/992</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07AAACR1234R1Z1</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v/>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Missing in Portal</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Invoice found in your books but absent from GST portal. May indicate delayed filing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>REL/MAY/992</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>07AAACR1234R1Z1</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v/>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Missing in Portal</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Invoice found in your books but absent from GST portal. May indicate delayed filing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>MISC/882</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>07AAACR1234R1Z1</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C10" s="2" t="n">
         <v>15000</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D10" s="2" t="n">
         <v>15000</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E10" s="2" t="n">
         <v>1800</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F10" s="2" t="n">
         <v>1800</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>Missing in Books</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>GST portal has this invoice but it has not been uploaded to the system.</t>
         </is>
@@ -967,7 +1279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -993,7 +1305,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -1003,37 +1315,27 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>21862</v>
+        <v>21886</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Status: Matched</t>
+          <t>Status: Mismatch</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Status: Mismatch</t>
+          <t>Status: Missing in Portal</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Status: Missing in Portal</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>